<commit_message>
02/04/2026 - MiniFix Se agrego la letra de candidatura a los reportes de empate de las COPACO
</commit_message>
<xml_diff>
--- a/plantillas/eleccion/Candidaturas_Empate.xlsx
+++ b/plantillas/eleccion/Candidaturas_Empate.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Visual Studio Code\NodeJS\SIVACC\plantillas\eleccion\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MrLuisKiller\Documents\Visual Studio Code\NodeJS\SIVACC\plantillas\eleccion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F33677D6-2CBC-4591-875E-EE3BE7A09C5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CED7BD78-28C6-4DE2-9390-A6CDC9ED184A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A40D9A0D-00B8-48B3-861D-4036705B821F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A40D9A0D-00B8-48B3-861D-4036705B821F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>Demarcación Territorial</t>
   </si>
@@ -60,13 +60,16 @@
   </si>
   <si>
     <t>Distrito</t>
+  </si>
+  <si>
+    <t>Letra(s) de Candidatura</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -101,6 +104,12 @@
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FFFF0000"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="3">
@@ -144,7 +153,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -166,6 +175,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -501,48 +513,52 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F3169C1-B902-4DC8-B58E-41F28DE01DBD}">
-  <dimension ref="A2:F11"/>
+  <dimension ref="A2:G11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.7109375" customWidth="1"/>
     <col min="2" max="2" width="30.7109375" customWidth="1"/>
     <col min="3" max="3" width="20.7109375" customWidth="1"/>
     <col min="4" max="4" width="35.7109375" customWidth="1"/>
-    <col min="5" max="5" width="45.7109375" customWidth="1"/>
-    <col min="6" max="6" width="30.7109375" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" customWidth="1"/>
+    <col min="6" max="6" width="45.7109375" customWidth="1"/>
+    <col min="7" max="7" width="30.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:6" ht="20.25" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="20.25" x14ac:dyDescent="0.25">
       <c r="A2" s="3"/>
       <c r="B2" s="3"/>
     </row>
-    <row r="3" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5"/>
       <c r="B3" s="5"/>
     </row>
-    <row r="5" spans="1:6" ht="18" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" ht="18" x14ac:dyDescent="0.25">
       <c r="A5" s="4"/>
       <c r="B5" s="4"/>
     </row>
-    <row r="6" spans="1:6" ht="18" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="18" x14ac:dyDescent="0.25">
       <c r="A6" s="4"/>
       <c r="B6" s="4"/>
     </row>
-    <row r="8" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="6"/>
       <c r="B8" s="6"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="7" t="s">
+      <c r="F8" s="2"/>
+      <c r="G8" s="7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="E9" s="2"/>
-      <c r="F9" s="7" t="s">
+    <row r="9" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="F9" s="2"/>
+      <c r="G9" s="7" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E10" s="8"/>
+    </row>
+    <row r="11" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>7</v>
       </c>
@@ -556,13 +572,17 @@
         <v>2</v>
       </c>
       <c r="E11" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F11" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="G11" s="1" t="s">
         <v>4</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>